<commit_message>
Split transcription scoring and verify seed data on launch
</commit_message>
<xml_diff>
--- a/PromptGradeApp/Defaults/Model_Testing_Rubric.xlsx
+++ b/PromptGradeApp/Defaults/Model_Testing_Rubric.xlsx
@@ -1984,9 +1984,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I48"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" ns3:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -1996,7 +1996,7 @@
     <col min="6" max="9" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="33.75" customHeight="1" ns3:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>19</v>
       </c>
@@ -2008,7 +2008,7 @@
       <c r="G1" s="3"/>
       <c r="H1" s="3"/>
     </row>
-    <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="30" customHeight="1" ns3:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>20</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A3" s="12" t="s">
         <v>29</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A4" s="12" t="s">
         <v>37</v>
       </c>
@@ -2095,7 +2095,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>44</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A6" s="12" t="s">
         <v>51</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A7" s="12" t="s">
         <v>59</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="57" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="57" ns3:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>66</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>73</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A10" s="12" t="s">
         <v>349</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="102.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="102.6" ns3:dyDescent="0.3">
       <c r="A11" s="12" t="s">
         <v>356</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="45.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="45.6" ns3:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>357</v>
       </c>
@@ -2327,7 +2327,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A13" s="12" t="s">
         <v>363</v>
       </c>
@@ -2356,7 +2356,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="45.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="45.6" ns3:dyDescent="0.3">
       <c r="A14" s="12" t="s">
         <v>367</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>80</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A16" s="12" t="s">
         <v>88</v>
       </c>
@@ -2443,7 +2443,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A17" s="12" t="s">
         <v>95</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A18" s="12" t="s">
         <v>102</v>
       </c>
@@ -2501,7 +2501,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>109</v>
       </c>
@@ -2530,7 +2530,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A20" s="12" t="s">
         <v>116</v>
       </c>
@@ -2559,7 +2559,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A21" s="12" t="s">
         <v>122</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A22" s="12" t="s">
         <v>129</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A23" s="12" t="s">
         <v>136</v>
       </c>
@@ -2646,7 +2646,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A24" s="12" t="s">
         <v>144</v>
       </c>
@@ -2675,7 +2675,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>151</v>
       </c>
@@ -2704,7 +2704,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A26" s="12" t="s">
         <v>158</v>
       </c>
@@ -2733,18 +2733,20 @@
         <v>164</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A27" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B27" s="13" t="s">
-        <v>166</v>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Transcription</t>
+        </is>
       </c>
       <c r="C27" s="13" t="s">
         <v>167</v>
       </c>
       <c r="D27" s="14">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>168</v>
@@ -2762,7 +2764,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A28" s="12" t="s">
         <v>173</v>
       </c>
@@ -2773,7 +2775,7 @@
         <v>174</v>
       </c>
       <c r="D28" s="14">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="E28" s="13" t="s">
         <v>175</v>
@@ -2791,7 +2793,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A29" s="12" t="s">
         <v>180</v>
       </c>
@@ -2802,7 +2804,7 @@
         <v>181</v>
       </c>
       <c r="D29" s="14">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E29" s="13" t="s">
         <v>182</v>
@@ -2820,7 +2822,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A30" s="12" t="s">
         <v>187</v>
       </c>
@@ -2831,7 +2833,7 @@
         <v>188</v>
       </c>
       <c r="D30" s="14">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E30" s="13" t="s">
         <v>189</v>
@@ -2849,7 +2851,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A31" s="12" t="s">
         <v>194</v>
       </c>
@@ -2878,7 +2880,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A32" s="12" t="s">
         <v>202</v>
       </c>
@@ -2907,7 +2909,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A33" s="12" t="s">
         <v>209</v>
       </c>
@@ -2936,7 +2938,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A34" s="12" t="s">
         <v>217</v>
       </c>
@@ -2965,7 +2967,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A35" s="12" t="s">
         <v>223</v>
       </c>
@@ -2994,7 +2996,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A36" s="12" t="s">
         <v>230</v>
       </c>
@@ -3023,7 +3025,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A37" s="12" t="s">
         <v>237</v>
       </c>
@@ -3052,7 +3054,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A38" s="12" t="s">
         <v>244</v>
       </c>
@@ -3081,7 +3083,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A39" s="12" t="s">
         <v>249</v>
       </c>
@@ -3110,7 +3112,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A40" s="12" t="s">
         <v>255</v>
       </c>
@@ -3139,7 +3141,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A41" s="12" t="s">
         <v>261</v>
       </c>
@@ -3168,7 +3170,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A42" s="12" t="s">
         <v>269</v>
       </c>
@@ -3197,7 +3199,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A43" s="12" t="s">
         <v>276</v>
       </c>
@@ -3226,7 +3228,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="34.200000000000003" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" ht="34.200000000000003" ns3:dyDescent="0.3">
       <c r="A44" s="38" t="s">
         <v>373</v>
       </c>
@@ -3255,7 +3257,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" ht="22.8" ns3:dyDescent="0.3">
       <c r="A45" s="38" t="s">
         <v>374</v>
       </c>
@@ -3284,7 +3286,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="45.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" ht="45.6" ns3:dyDescent="0.3">
       <c r="A46" s="38" t="s">
         <v>375</v>
       </c>
@@ -3310,7 +3312,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="45.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" ht="45.6" ns3:dyDescent="0.3">
       <c r="A47" s="38" t="s">
         <v>376</v>
       </c>
@@ -3336,7 +3338,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="45.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="45.6" ns3:dyDescent="0.3">
       <c r="A48" s="38" t="s">
         <v>377</v>
       </c>

</xml_diff>